<commit_message>
feat(seo): 50 unique bespoke titles and distinct 13-tag SEO stacks for sardine tin cases
</commit_message>
<xml_diff>
--- a/output/sardine_tin_market_intelligence_100_designs.xlsx
+++ b/output/sardine_tin_market_intelligence_100_designs.xlsx
@@ -6700,15 +6700,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #1, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Porto Classic Sardinhas Phone Case, Portuguese Azulejo Tile Fish Can Cover iPhone 16 Pro Max Samsung S25 Ultra MagSafe</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>portuguese sardine phone case, azulejo tile phone case, lisbon sardinha case, vintage conservas cover, portuguese tile case, mediterranean phone case, blue and white tile case, canned fish phone case, iphone 16 pro max case, samsung s25 ultra tough cover, magsafe phone case, aesthetic food phone case, unique foodie gift</t>
+          <t>portuguese sardine, azulejo tile case, lisbon sardinha, vintage conservas, portuguese tile, mediterranean phone, blue white tile, canned fish case, iphone 16 pro max, samsung s25 ultra, magsafe case, foodie gift for her, lisbon souvenir</t>
         </is>
       </c>
     </row>
@@ -6718,15 +6718,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #2, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Galo de Barcelos Portuguese Phone Case, Vintage Rooster Spicy Sardine Tin Cover iPhone 16 15 Pro Max Galaxy S25 MagSafe</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>french sardine phone case, vintage french tin case, concarneau seafood case, art nouveau fish case, parisian bistro phone case, vintage packaging case, belle epoque phone cover, french food phone case, iphone 16 case, samsung galaxy tough case, gourmet food gift, aesthetic mirror selfie case, retro kitchen phone cover</t>
+          <t>galo de barcelos, portuguese rooster, spicy sardine case, portugal folk art, piri piri sardine, lisbon fish can, portuguese gift, vintage food can, iphone 16 case, galaxy s25 cover, magsafe tough case, retro kitchen art, folk illustration</t>
         </is>
       </c>
     </row>
@@ -6736,15 +6736,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #3, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Algarve Fisherman Morning Haul Sardines Phone Case, Atlantic Ocean Coastal Catch Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>sardine tin phone case, coastal grandmother phone case, nantucket lobster phone case, watercolor fish tin case, preppy coastal phone, blue hydrangea phone case, beach cottage phone cover, cape cod seafood case, iphone 16 pro max, samsung s24 ultra case, magsafe tough case, vintage seafood art, summer holiday gift</t>
+          <t>algarve phone case, fisherman case, atlantic sardine, ocean fish tin, portugal beach case, vintage maritime, nautical phone case, coastal gift, iphone 16 pro max, samsung s24 ultra, seafood can cover, mens nautical gift, tough phone case</t>
         </is>
       </c>
     </row>
@@ -6754,15 +6754,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #4, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Lisbon Tram 28 Sardine Express Phone Case, Vintage Yellow Trolley Tin Cover iPhone 16 15 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>tomato girl phone case, aperol spritz sardine case, euro summer phone case, amalfi coast fish case, mediterranean picnic case, lemon sardine phone cover, italian vacation phone case, coastal aesthetic case, iphone 15 pro max case, galaxy s25 tough cover, cute food phone case, aesthetic brunch phone, trendy summer gift</t>
+          <t>tram 28 phone case, lisbon tram case, yellow trolley tin, portugal travel, lisbon wanderlust, vintage transit, portuguese souvenir, canned fish look, iphone 16 pro, galaxy s25 ultra, europe travel gift, aesthetic food cover, magsafe phone case</t>
         </is>
       </c>
     </row>
@@ -6772,15 +6772,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #5, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Azulejo Ceramic Tile Sardine Mosaic Phone Case, Cobalt Blue Delft Pilchard Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>caviar tin phone case, luxury oyster phone case, vintage champagne tin case, old money aesthetic case, gourmet seafood phone, royal sturgeon phone cover, black and gold phone case, oyster shell phone case, iphone 16 pro max case, samsung s25 ultra cover, elegant luxury phone case, fine dining food gift, quiet luxury tech</t>
+          <t>azulejo mosaic case, blue and white tile, ceramic pattern case, delft blue phone, geometric fish case, mediterranean decor, lisbon tiles, sardine art cover, iphone 16 pro max, samsung s25 tough, artistic phone case, interior design gift, magsafe accessory</t>
         </is>
       </c>
     </row>
@@ -6790,15 +6790,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #6, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Les Sardines de Bretagne Phone Case, Vintage French Concarneau Seafood Tin Cover iPhone 16 Pro Max Samsung S25 Ultra</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>cat sardine phone case, funny cat fish tin case, cat stealing sardine case, cute cat food case, quirky cat phone cover, orange tabby phone case, black cat phone case, kitten sardine tin bed, iphone 16 case, samsung galaxy s24 cover, funny animal phone case, cat lover gift for her, aesthetic meme phone case</t>
+          <t>french sardine case, bretagne seafood, vintage french tin, concarneau fish can, belle epoque case, french country art, parisian aesthetic, gourmet seafood, iphone 16 pro max, samsung s25 cover, magsafe tough case, francophile gift, french kitchen decor</t>
         </is>
       </c>
     </row>
@@ -6808,15 +6808,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #7, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Le Petit Pecheur Nantes Sardines Phone Case, Vintage French Fisherman Child Tin Cover iPhone 16 15 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>spanish tapas phone case, conservas collage case, maximalist seafood case, razor clam tin case, retro bar phone case, spanish mussel phone cover, madrid food aesthetic, tapas lover phone case, iphone 16 pro case, samsung s25 ultra tough cover, colorful food pattern, indie art phone case, bold kitchen art cover</t>
+          <t>le petit pecheur, french fisherman, retro french label, nantes sardine tin, yellow slicker art, storybook phone case, vintage food label, cute french cover, iphone 16 case, galaxy s25 ultra, nostalgic gift, french illustration, magsafe tough cover</t>
         </is>
       </c>
     </row>
@@ -6826,15 +6826,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #8, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Sardines Royales Provencal Herbs Phone Case, Vintage French Lavender Olive Oil Can iPhone 16 Pro Max Samsung S25 Ultra</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>nordic sardine phone case, scandinavian fish tin case, copenhagen aesthetic phone, smoked sprat case, minimalist fish case, danish smorrebrod phone case, baltic herring phone cover, clean scandi phone case, iphone 16 case, samsung s24 case, modern minimalist phone case, architectural graphic case, aesthetic gift</t>
+          <t>provencal sardine, french herb tin, provence lavender, gourmet french food, botanical tin case, olive oil seafood, french cottagecore, vintage apothecary, iphone 16 pro max, samsung s25 tough, magsafe case, aesthetic foodie, french lifestyle</t>
         </is>
       </c>
     </row>
@@ -6844,15 +6844,15 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #9, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Le Bistrot Parisien Sardines Phone Case, Vintage Marble Bistro Chablis Wine Can Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>yacht club phone case, vintage nautical tin case, saint tropez seafood case, riviera sailing phone case, maritime provisions case, monaco grand prix phone, sailing flag phone case, boat lover phone cover, iphone 16 pro max case, samsung s25 tough case, preppy nautical gift, coastal aesthetic phone, magsafe cover</t>
+          <t>parisian bistro, french cafe case, wine and sardines, chablis wine art, bistro chalkboard, paris lifestyle, retro restaurant, french food gift, iphone 16 pro max, galaxy s25 cover, magsafe tough case, mirror selfie case, foodcore aesthetic</t>
         </is>
       </c>
     </row>
@@ -6862,15 +6862,15 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vintage Portuguese Sardine Tin Phone Case #10, Azulejo Blue Tile Conservas Cover for iPhone 16 15 14 Pro Max Samsung S25 Ultra MagSafe</t>
+          <t>Le Chat Gourmand French Bistro Cat Phone Case, Vintage Art Nouveau Steinlen Sardine Can iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3d sardine tin phone case, peel back tin phone case, metal sardine can case, realistic sardine can case, illusion food case, open tin can phone cover, funny food phone case, realistic 3d food case, iphone 16 pro max case, samsung s25 ultra cover, novelty phone case, viral tiktok phone case, conversation starter</t>
+          <t>le chat noir case, french bistro cat, black cat sardine, art nouveau phone, steinlen cat art, whimsical cat gift, vintage cabaret, parisian cat cover, iphone 16 pro max, samsung s25 ultra, cat lover phone case, cute kitten tech, magsafe phone cover</t>
         </is>
       </c>
     </row>
@@ -6880,15 +6880,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #11, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Nantucket Harbor Blue Hydrangea Sardine Tin Phone Case, Coastal Grandmother Seafood Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>portuguese sardine phone case, azulejo tile phone case, lisbon sardinha case, vintage conservas cover, portuguese tile case, mediterranean phone case, blue and white tile case, canned fish phone case, iphone 16 pro max case, samsung s25 ultra tough cover, magsafe phone case, aesthetic food phone case, unique foodie gift</t>
+          <t>nantucket phone case, coastal grandmother, hydrangea sardine, blue hydrangea case, preppy coastal gift, beach cottage decor, cape cod seafood, watercolor fish can, iphone 16 pro max, samsung s25 tough, magsafe cover, summer beach tech, grandmillennial</t>
         </is>
       </c>
     </row>
@@ -6898,15 +6898,15 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #12, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Cape Cod Bay Fishmonger Sardine Phone Case, Weathered Wooden Seafood Sign Cover iPhone 16 15 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>french sardine phone case, vintage french tin case, concarneau seafood case, art nouveau fish case, parisian bistro phone case, vintage packaging case, belle epoque phone cover, french food phone case, iphone 16 case, samsung galaxy tough case, gourmet food gift, aesthetic mirror selfie case, retro kitchen phone cover</t>
+          <t>cape cod phone case, fishmonger sign, weathered coastal, new england seafood, driftwood aesthetic, vintage harbor art, beach house style, seafood market case, iphone 16 pro, galaxy s25 ultra, coastal gift for him, rustic nautical, magsafe phone cover</t>
         </is>
       </c>
     </row>
@@ -6916,15 +6916,15 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #13, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Martha's Vineyard Striped Sailboat Sardine Case, Preppy Navy Cabana Seafood Can Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>sardine tin phone case, coastal grandmother phone case, nantucket lobster phone case, watercolor fish tin case, preppy coastal phone, blue hydrangea phone case, beach cottage phone cover, cape cod seafood case, iphone 16 pro max, samsung s24 ultra case, magsafe tough case, vintage seafood art, summer holiday gift</t>
+          <t>marthas vineyard, preppy nautical, striped phone case, sailboat sardine, yachting aesthetic, old money summer, navy cabana stripe, new england preppy, iphone 16 pro max, samsung s25 tough, coastal boy aesthetic, preppy gift for her, magsafe tough case</t>
         </is>
       </c>
     </row>
@@ -6934,15 +6934,15 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #14, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Coastal Picnic Gingham Tablecloth Sardines Case, Sourdough Bread Seafood Feast Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>tomato girl phone case, aperol spritz sardine case, euro summer phone case, amalfi coast fish case, mediterranean picnic case, lemon sardine phone cover, italian vacation phone case, coastal aesthetic case, iphone 15 pro max case, galaxy s25 tough cover, cute food phone case, aesthetic brunch phone, trendy summer gift</t>
+          <t>gingham picnic case, sourdough sardines, coastal picnic, cottagecore food, red gingham pattern, aesthetic lunch art, foodie picnic cover, summer picnic gift, iphone 16 pro max, samsung s25 ultra, magsafe phone case, mirror selfie tech, cute food cover</t>
         </is>
       </c>
     </row>
@@ -6952,15 +6952,15 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #15, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Block Island Summer Catch Shells Sardine Case, Pastel Sea Glass Beach Scallop Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>caviar tin phone case, luxury oyster phone case, vintage champagne tin case, old money aesthetic case, gourmet seafood phone, royal sturgeon phone cover, black and gold phone case, oyster shell phone case, iphone 16 pro max case, samsung s25 ultra cover, elegant luxury phone case, fine dining food gift, quiet luxury tech</t>
+          <t>block island case, sea glass phone, scallop shell art, pastel coastal, beachcomber gift, soft ocean aesthetic, seashell sardine tin, island summer tech, iphone 16 pro max, samsung s25 tough, magsafe accessory, coastal chic cover, mermaid core phone</t>
         </is>
       </c>
     </row>
@@ -6970,15 +6970,15 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #16, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Amalfi Coast Lemon Grove Sardines Phone Case, Mediterranean Citrus Olive Oil Tin Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>cat sardine phone case, funny cat fish tin case, cat stealing sardine case, cute cat food case, quirky cat phone cover, orange tabby phone case, black cat phone case, kitten sardine tin bed, iphone 16 case, samsung galaxy s24 cover, funny animal phone case, cat lover gift for her, aesthetic meme phone case</t>
+          <t>amalfi lemon case, tomato girl summer, italian sardine, amalfi coast decor, mediterranean lemon, euro summer case, positanovibes, citrus food art, iphone 16 pro max, samsung s25 ultra, magsafe tough case, cute foodie gift, summer vacation tech</t>
         </is>
       </c>
     </row>
@@ -6988,15 +6988,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #17, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Positano Cliffside Aperitivo Spritz Phone Case, Italian Vacation Sardine Tapas Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>spanish tapas phone case, conservas collage case, maximalist seafood case, razor clam tin case, retro bar phone case, spanish mussel phone cover, madrid food aesthetic, tapas lover phone case, iphone 16 pro case, samsung s25 ultra tough cover, colorful food pattern, indie art phone case, bold kitchen art cover</t>
+          <t>positano phone case, aperol spritz case, italian holiday, aperitivo hour, cliffside village, euro summer aesthetic, cocktail phone case, terracotta sunset, iphone 16 pro max, galaxy s25 tough, italy travel souvenir, magsafe cover, aesthetic summer</t>
         </is>
       </c>
     </row>
@@ -7006,15 +7006,15 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #18, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Capri Blue Grotto Sardine Mosaic Phone Case, Luminous Azure Sea Mediterranean Cover iPhone 16 Pro Max Samsung S25 Ultra</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>nordic sardine phone case, scandinavian fish tin case, copenhagen aesthetic phone, smoked sprat case, minimalist fish case, danish smorrebrod phone case, baltic herring phone cover, clean scandi phone case, iphone 16 case, samsung s24 case, modern minimalist phone case, architectural graphic case, aesthetic gift</t>
+          <t>capri blue grotto, italian island case, azure sea mosaic, luminous blue phone, mediterranean grotto, luxury travel tech, capri vacation gift, vibrant ocean case, iphone 16 pro max, samsung s25 tough, magsafe phone cover, island aesthetic, deep blue cover</t>
         </is>
       </c>
     </row>
@@ -7024,15 +7024,15 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #19, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Tomato Girl Summer Heirloom Toast Phone Case, Sourdough Sliced Tomato Sardine Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>yacht club phone case, vintage nautical tin case, saint tropez seafood case, riviera sailing phone case, maritime provisions case, monaco grand prix phone, sailing flag phone case, boat lover phone cover, iphone 16 pro max case, samsung s25 tough case, preppy nautical gift, coastal aesthetic phone, magsafe cover</t>
+          <t>tomato girl aesthetic, heirloom tomato, sardine toast case, food aesthetic tech, sourdough toast art, dopamine food decor, trendy foodcore, tiktok viral case, iphone 16 pro max, galaxy s25 cover, magsafe phone case, cool girl aesthetic, foodie gift</t>
         </is>
       </c>
     </row>
@@ -7042,15 +7042,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>French Seafood Tin Phone Case #20, Vintage Brittany Sardine Can Belle Époque Aesthetic for iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Sicilian Blood Orange Chili Sardines Phone Case, Southern Italy Folk Ceramic Can Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3d sardine tin phone case, peel back tin phone case, metal sardine can case, realistic sardine can case, illusion food case, open tin can phone cover, funny food phone case, realistic 3d food case, iphone 16 pro max case, samsung s25 ultra cover, novelty phone case, viral tiktok phone case, conversation starter</t>
+          <t>sicilian sardine, blood orange phone, spicy chili sardine, sicily folk ceramic, bold italian art, southern italy case, fiery food decor, vintage cannery, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, colorful phone case, bold graphic cover</t>
         </is>
       </c>
     </row>
@@ -7060,15 +7060,15 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #21, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Petrossian Style Imperial Beluga Caviar Phone Case, Old Money Gilded Black Sturgeon Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>portuguese sardine phone case, azulejo tile phone case, lisbon sardinha case, vintage conservas cover, portuguese tile case, mediterranean phone case, blue and white tile case, canned fish phone case, iphone 16 pro max case, samsung s25 ultra tough cover, magsafe phone case, aesthetic food phone case, unique foodie gift</t>
+          <t>caviar tin phone, beluga caviar case, old money aesthetic, quiet luxury tech, gilded sturgeon art, black gold phone, imperial gourmet, luxury foodie gift, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, sophisticated cover, fine dining merch</t>
         </is>
       </c>
     </row>
@@ -7078,15 +7078,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #22, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Normandy Raw Oyster Bar Mignonette Phone Case, Half Shell Oyster Lemon Platter Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>french sardine phone case, vintage french tin case, concarneau seafood case, art nouveau fish case, parisian bistro phone case, vintage packaging case, belle epoque phone cover, french food phone case, iphone 16 case, samsung galaxy tough case, gourmet food gift, aesthetic mirror selfie case, retro kitchen phone cover</t>
+          <t>oyster phone case, raw bar seafood, normandy oyster, mignonette lemon, half shell oyster, oyster shell aesthetic, coastal gourmet, seafood platter art, iphone 16 pro max, samsung s25 tough, magsafe phone case, preppy seafood gift, beach food cover</t>
         </is>
       </c>
     </row>
@@ -7096,15 +7096,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #23, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Saint-Malo Wild Blue Lobster Cannery Phone Case, French Brittany Heraldic Seafood Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>sardine tin phone case, coastal grandmother phone case, nantucket lobster phone case, watercolor fish tin case, preppy coastal phone, blue hydrangea phone case, beach cottage phone cover, cape cod seafood case, iphone 16 pro max, samsung s24 ultra case, magsafe tough case, vintage seafood art, summer holiday gift</t>
+          <t>blue lobster case, french lobster tin, saint malo seafood, bretagne blue lobster, heraldic crest art, gilded brass navy, luxury crustacean, vintage french food, iphone 16 pro max, galaxy s25 ultra, magsafe tough case, mens nautical gift, quiet luxury phone</t>
         </is>
       </c>
     </row>
@@ -7114,15 +7114,15 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #24, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Art Deco Royal Sturgeon Champagne Caviar Case, Gilded Gold Geometric Seafood Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>tomato girl phone case, aperol spritz sardine case, euro summer phone case, amalfi coast fish case, mediterranean picnic case, lemon sardine phone cover, italian vacation phone case, coastal aesthetic case, iphone 15 pro max case, galaxy s25 tough cover, cute food phone case, aesthetic brunch phone, trendy summer gift</t>
+          <t>champagne caviar case, art deco seafood, royal sturgeon art, gilded gold case, geometric luxury, 1920s vintage glam, quiet luxury tech, celebration gift, iphone 16 pro max, samsung s25 tough, magsafe phone cover, black tie aesthetic, high end phone case</t>
         </is>
       </c>
     </row>
@@ -7132,15 +7132,15 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #25, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Stained Glass Oyster Pearl Suncatcher Phone Case, Iridescent Scallop Cathedral Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>caviar tin phone case, luxury oyster phone case, vintage champagne tin case, old money aesthetic case, gourmet seafood phone, royal sturgeon phone cover, black and gold phone case, oyster shell phone case, iphone 16 pro max case, samsung s25 ultra cover, elegant luxury phone case, fine dining food gift, quiet luxury tech</t>
+          <t>stained glass oyster, pearl shell phone, iridescent sea case, suncatcher phone cover, cathedral glass art, ocean jewel case, pastel refraction, scallop pearl gift, iphone 16 pro max, samsung s25 ultra, magsafe tough case, mermaidcore case, aesthetic ocean</t>
         </is>
       </c>
     </row>
@@ -7150,15 +7150,15 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #26, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>The Midnight Sardine Burglar Black Cat Phone Case, Mischievous Kitty Stealing Fish Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>cat sardine phone case, funny cat fish tin case, cat stealing sardine case, cute cat food case, quirky cat phone cover, orange tabby phone case, black cat phone case, kitten sardine tin bed, iphone 16 case, samsung galaxy s24 cover, funny animal phone case, cat lover gift for her, aesthetic meme phone case</t>
+          <t>black cat sardine, cat burglar phone, mischievous kitten, funny cat phone case, cat stealing fish, midnight black cat, quirky animal case, cat mom aesthetic, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, cute pet lover gift, humorous phone cover</t>
         </is>
       </c>
     </row>
@@ -7168,15 +7168,15 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #27, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Orange Tabby Sleeping in Sardine Tin Bed Phone Case, Cozy Kawaii Cat Can Nap Cover iPhone 16 15 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>spanish tapas phone case, conservas collage case, maximalist seafood case, razor clam tin case, retro bar phone case, spanish mussel phone cover, madrid food aesthetic, tapas lover phone case, iphone 16 pro case, samsung s25 ultra tough cover, colorful food pattern, indie art phone case, bold kitchen art cover</t>
+          <t>orange tabby case, cat in sardine bed, cozy kawaii cat, sleeping cat phone, cute kitten in tin, ginger cat aesthetic, whimsical pet art, cat mom gift for her, iphone 16 case, galaxy s25 ultra, magsafe tough case, snuggly cat cover, kawaii animal case</t>
         </is>
       </c>
     </row>
@@ -7186,15 +7186,15 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #28, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Cat with Stolen Sardine Zero Regrets Phone Case, Funny Fluffy White Kitten Fish Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>nordic sardine phone case, scandinavian fish tin case, copenhagen aesthetic phone, smoked sprat case, minimalist fish case, danish smorrebrod phone case, baltic herring phone cover, clean scandi phone case, iphone 16 case, samsung s24 case, modern minimalist phone case, architectural graphic case, aesthetic gift</t>
+          <t>cat zero regrets, stolen sardine case, funny meme cat, fluffy white kitten, viral cat humor, quirky pop art cat, dopamine pet merch, proud cat thief, iphone 16 pro max, samsung s25 tough, magsafe phone cover, silly animal gift, trending pet case</t>
         </is>
       </c>
     </row>
@@ -7204,15 +7204,15 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #29, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Tuxedo Cat Waiter French Sardine Tin Phone Case, Dapper Bowtie Kitty Bistro Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>yacht club phone case, vintage nautical tin case, saint tropez seafood case, riviera sailing phone case, maritime provisions case, monaco grand prix phone, sailing flag phone case, boat lover phone cover, iphone 16 pro max case, samsung s25 tough case, preppy nautical gift, coastal aesthetic phone, magsafe cover</t>
+          <t>tuxedo cat phone, dapper cat waiter, french bistro kitty, bowtie cat art, vintage cartoon cat, sophisticated pet, quirky cat food case, cat lover phone cover, iphone 16 pro max, galaxy s25 tough, magsafe phone case, whimsical pet gift, black and white cat</t>
         </is>
       </c>
     </row>
@@ -7222,15 +7222,15 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Coastal Grandmother Sardine Tin Phone Case #30, Nantucket Blue Hydrangea Watercolor Fish Cover iPhone 16 Pro Max Samsung S24</t>
+          <t>Curious Cat Peeking Through Peeled Tin Foil Lid Case, Cute Kitty Paws Metal Can Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3d sardine tin phone case, peel back tin phone case, metal sardine can case, realistic sardine can case, illusion food case, open tin can phone cover, funny food phone case, realistic 3d food case, iphone 16 pro max case, samsung s25 ultra cover, novelty phone case, viral tiktok phone case, conversation starter</t>
+          <t>cat peeking tin lid, peeled foil cat, curious kitten paws, cutout paper cat, funny peekaboo cat, minimalist cat art, quirky animal tech, cat lover accessory, iphone 16 pro max, samsung s25 ultra, magsafe tough case, playful pet cover, viral animal phone</t>
         </is>
       </c>
     </row>
@@ -7240,15 +7240,15 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #31, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Madrid Tapas Bar Conservas Wall Collage Phone Case, Maximalist Spanish Seafood Can Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>portuguese sardine phone case, azulejo tile phone case, lisbon sardinha case, vintage conservas cover, portuguese tile case, mediterranean phone case, blue and white tile case, canned fish phone case, iphone 16 pro max case, samsung s25 ultra tough cover, magsafe phone case, aesthetic food phone case, unique foodie gift</t>
+          <t>madrid tapas case, conservas collage, spanish seafood wall, maximalist phone case, tapas bar aesthetic, vintage spanish cans, colorful food decor, spain travel souvenir, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, graphic designer gift, pop art phone case</t>
         </is>
       </c>
     </row>
@@ -7258,15 +7258,15 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #32, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Galician Spicy Mussels Escabeche Tin Phone Case, Vintage Spanish Conservas Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>french sardine phone case, vintage french tin case, concarneau seafood case, art nouveau fish case, parisian bistro phone case, vintage packaging case, belle epoque phone cover, french food phone case, iphone 16 case, samsung galaxy tough case, gourmet food gift, aesthetic mirror selfie case, retro kitchen phone cover</t>
+          <t>spanish mussels case, escabeche tin cover, galician seafood, spicy paprika fish, vintage spanish label, bold orange phone, foodie phone case, conservas collector, iphone 16 pro max, galaxy s25 tough, magsafe phone cover, spain foodie gift, bold kitchen art</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #33, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Barcelona Vermouth Hour Sardines Gilda Skewer Case, Retro Spanish Bodega Tapas Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>sardine tin phone case, coastal grandmother phone case, nantucket lobster phone case, watercolor fish tin case, preppy coastal phone, blue hydrangea phone case, beach cottage phone cover, cape cod seafood case, iphone 16 pro max, samsung s24 ultra case, magsafe tough case, vintage seafood art, summer holiday gift</t>
+          <t>barcelona tapas, vermouth hour case, gilda skewer art, spanish bodega cover, mid century bar art, olive anchovy skewer, catalonia travel, cocktail hour phone, iphone 16 pro max, samsung s25 tough, magsafe phone case, retro foodie merch, spanish food decor</t>
         </is>
       </c>
     </row>
@@ -7294,15 +7294,15 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #34, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Pulpo a la Gallega Octopus Paprika Tin Phone Case, Woodcut Spanish Seafood Can Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>tomato girl phone case, aperol spritz sardine case, euro summer phone case, amalfi coast fish case, mediterranean picnic case, lemon sardine phone cover, italian vacation phone case, coastal aesthetic case, iphone 15 pro max case, galaxy s25 tough cover, cute food phone case, aesthetic brunch phone, trendy summer gift</t>
+          <t>pulpo gallego case, octopus phone case, paprika octopus tin, woodcut seafood art, camino souvenir, spanish octopus cover, bold ocean animal, coarse sea salt art, iphone 16 pro max, galaxy s25 ultra, magsafe tough case, adventurous foodie, ocean creature tech</t>
         </is>
       </c>
     </row>
@@ -7312,15 +7312,15 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #35, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Seville Flamenco Dancer Gilded Sardines Phone Case, Vintage Andalusian Scarlet Polka Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>caviar tin phone case, luxury oyster phone case, vintage champagne tin case, old money aesthetic case, gourmet seafood phone, royal sturgeon phone cover, black and gold phone case, oyster shell phone case, iphone 16 pro max case, samsung s25 ultra cover, elegant luxury phone case, fine dining food gift, quiet luxury tech</t>
+          <t>seville flamenco, andalusian phone, spanish dancer art, scarlet red polka, castanet seafood, vintage andalucia, romantic spanish cover, spain culture gift, iphone 16 pro max, samsung s25 tough, magsafe phone case, dramatic art case, flamenco lover gift</t>
         </is>
       </c>
     </row>
@@ -7330,15 +7330,15 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #36, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Copenhagen Smoked Herring Dark Rye Bread Phone Case, Minimalist Danish Smorrebrod Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>cat sardine phone case, funny cat fish tin case, cat stealing sardine case, cute cat food case, quirky cat phone cover, orange tabby phone case, black cat phone case, kitten sardine tin bed, iphone 16 case, samsung galaxy s24 cover, funny animal phone case, cat lover gift for her, aesthetic meme phone case</t>
+          <t>copenhagen phone, danish smorrebrod, smoked herring case, scandi minimalist, dark rye bread art, nordic food decor, copenhagen style, clean line art phone, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, architectural gift, nordic aesthetic</t>
         </is>
       </c>
     </row>
@@ -7348,15 +7348,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #37, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Baltic Sea Sprats Vintage Brass Tin Phone Case, Understated Scandi Typography Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>spanish tapas phone case, conservas collage case, maximalist seafood case, razor clam tin case, retro bar phone case, spanish mussel phone cover, madrid food aesthetic, tapas lover phone case, iphone 16 pro case, samsung s25 ultra tough cover, colorful food pattern, indie art phone case, bold kitchen art cover</t>
+          <t>baltic sprats case, scandi typography, brass tin phone, minimalist fish art, ostresjo brisling, dill green aesthetic, clean scandi cover, nordic tech case, iphone 16 pro max, galaxy s25 tough, magsafe phone case, swedish design gift, understated tech</t>
         </is>
       </c>
     </row>
@@ -7366,15 +7366,15 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #38, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Stockholm Archipelago Midsummer Herring Phone Case, Nordic Wildflower Flower Crown Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>nordic sardine phone case, scandinavian fish tin case, copenhagen aesthetic phone, smoked sprat case, minimalist fish case, danish smorrebrod phone case, baltic herring phone cover, clean scandi phone case, iphone 16 case, samsung s24 case, modern minimalist phone case, architectural graphic case, aesthetic gift</t>
+          <t>midsummer phone case, stockholm herring, swedish wildflower, flower crown phone, nordic summer art, archipelago boat, scandinavian holiday, sweden travel gift, iphone 16 pro max, samsung s25 ultra, magsafe tough case, floral ocean cover, scandi aesthetic</t>
         </is>
       </c>
     </row>
@@ -7384,15 +7384,15 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #39, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Norwegian Fjord Salmon Sardines Cannery Phone Case, Arctic Mountain Rorbu Cabin Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>yacht club phone case, vintage nautical tin case, saint tropez seafood case, riviera sailing phone case, maritime provisions case, monaco grand prix phone, sailing flag phone case, boat lover phone cover, iphone 16 pro max case, samsung s25 tough case, preppy nautical gift, coastal aesthetic phone, magsafe cover</t>
+          <t>norwegian fjord case, rorbu cabin phone, arctic ocean sardine, norway travel cover, snow mountain art, scandinavian export, rugged nordic phone, lofoten islands gift, iphone 16 pro max, galaxy s25 tough, magsafe phone cover, nordic wanderlust, outdoor adventurer</t>
         </is>
       </c>
     </row>
@@ -7402,15 +7402,15 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Euro Summer Tomato Girl Sardine Phone Case #40, Amalfi Lemon &amp; Aperitivo Spritz Mediterranean Cover iPhone 16 Samsung S25</t>
+          <t>Nordic Hygge Candlelight Winter Sardines Phone Case, Cozy Wool Knit Snacking Cover iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3d sardine tin phone case, peel back tin phone case, metal sardine can case, realistic sardine can case, illusion food case, open tin can phone cover, funny food phone case, realistic 3d food case, iphone 16 pro max case, samsung s25 ultra cover, novelty phone case, viral tiktok phone case, conversation starter</t>
+          <t>hygge phone case, nordic winter cozy, beeswax candle art, wool knit aesthetic, cozy lifestyle tech, winter snacking case, warm scandi cover, hygge gift for her, iphone 16 pro max, samsung s25 tough, magsafe phone case, snuggly winter phone, minimalist warmth</t>
         </is>
       </c>
     </row>
@@ -7420,15 +7420,15 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #41, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Monaco Yacht Club Grand Prix Sardine Provisions Case, Vintage Monte Carlo Regatta Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>portuguese sardine phone case, azulejo tile phone case, lisbon sardinha case, vintage conservas cover, portuguese tile case, mediterranean phone case, blue and white tile case, canned fish phone case, iphone 16 pro max case, samsung s25 ultra tough cover, magsafe phone case, aesthetic food phone case, unique foodie gift</t>
+          <t>monaco yacht case, grand prix phone, regatta flag cover, teak wood boat art, monte carlo luxury, vintage yacht club, french riviera tech, old money nautical, iphone 16 pro max, samsung s25 ultra, magsafe tough case, sailing captain gift, preppy maritime</t>
         </is>
       </c>
     </row>
@@ -7438,15 +7438,15 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #42, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Saint-Tropez Harbor Pastel Fishing Schooner Case, French Riviera Sunlit Sardine Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>french sardine phone case, vintage french tin case, concarneau seafood case, art nouveau fish case, parisian bistro phone case, vintage packaging case, belle epoque phone cover, french food phone case, iphone 16 case, samsung galaxy tough case, gourmet food gift, aesthetic mirror selfie case, retro kitchen phone cover</t>
+          <t>saint tropez case, french harbor boat, pastel fishing boat, french riviera cover, sunlit ocean art, coastal chic tech, port de st tropez, summer in france gift, iphone 16 pro max, galaxy s25 tough, magsafe phone cover, glamorous beach case, riviera holiday</t>
         </is>
       </c>
     </row>
@@ -7456,15 +7456,15 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #43, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Commodore Vintage Brass Compass Seafood Tin Case, Antique Maritime Navigation Chart iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>sardine tin phone case, coastal grandmother phone case, nantucket lobster phone case, watercolor fish tin case, preppy coastal phone, blue hydrangea phone case, beach cottage phone cover, cape cod seafood case, iphone 16 pro max, samsung s24 ultra case, magsafe tough case, vintage seafood art, summer holiday gift</t>
+          <t>brass compass case, nautical chart phone, vintage navigation, commodore yacht club, antique map seafood, sailor gift for him, brass cleat aesthetic, coastal mens tech, iphone 16 pro max, samsung s25 tough, magsafe phone case, traditional marine, ocean voyager</t>
         </is>
       </c>
     </row>
@@ -7474,15 +7474,15 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #44, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Classic Mahogany Riva Boat Lake Como Sardines Case, Italian Boating Chrome Marine Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>tomato girl phone case, aperol spritz sardine case, euro summer phone case, amalfi coast fish case, mediterranean picnic case, lemon sardine phone cover, italian vacation phone case, coastal aesthetic case, iphone 15 pro max case, galaxy s25 tough cover, cute food phone case, aesthetic brunch phone, trendy summer gift</t>
+          <t>riva boat phone case, lake como boating, italian yacht style, varnished mahogany, chrome marine cleat, quiet luxury boat, dolce vita aesthetic, lake como souvenir, iphone 16 pro max, galaxy s25 ultra, magsafe tough cover, gentlemans tech, italian elegance</t>
         </is>
       </c>
     </row>
@@ -7492,15 +7492,15 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #45, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Maritime Signal Flag Alphabet Sardine Yacht Case, Vintage Nautical Pennant Banner Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>caviar tin phone case, luxury oyster phone case, vintage champagne tin case, old money aesthetic case, gourmet seafood phone, royal sturgeon phone cover, black and gold phone case, oyster shell phone case, iphone 16 pro max case, samsung s25 ultra cover, elegant luxury phone case, fine dining food gift, quiet luxury tech</t>
+          <t>signal flag case, nautical alphabet, maritime pennants, sailing code cover, bold nautical flags, yachting preppy tech, ocean signal banner, boating gift for her, iphone 16 pro max, samsung s25 ultra, magsafe phone cover, preppy sailor case, coastal flag art</t>
         </is>
       </c>
     </row>
@@ -7510,15 +7510,15 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #46, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>The Open Can 3D Peel-Back Foil Sardine Phone Case, Realistic Metallic Lid Fish Illusion iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>cat sardine phone case, funny cat fish tin case, cat stealing sardine case, cute cat food case, quirky cat phone cover, orange tabby phone case, black cat phone case, kitten sardine tin bed, iphone 16 case, samsung galaxy s24 cover, funny animal phone case, cat lover gift for her, aesthetic meme phone case</t>
+          <t>3d sardine tin case, peel back tin lid, metal sardine can, optical illusion case, realistic fish can, open tin phone cover, viral tiktok gadget, conversation starter, iphone 16 pro max, samsung s25 ultra, magsafe tough cover, funny food novelty, hyperrealistic 3d</t>
         </is>
       </c>
     </row>
@@ -7528,15 +7528,15 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #47, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Embossed 24K Gold Royal Sardine Tin Phone Case, 3D Raised Metallic Relief Foil Cover iPhone 16 Pro Max Galaxy S25 Ultra</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>spanish tapas phone case, conservas collage case, maximalist seafood case, razor clam tin case, retro bar phone case, spanish mussel phone cover, madrid food aesthetic, tapas lover phone case, iphone 16 pro case, samsung s25 ultra tough cover, colorful food pattern, indie art phone case, bold kitchen art cover</t>
+          <t>gold sardine tin, embossed metal case, 3d royal fish can, metallic foil relief, antique gold lacquer, luxury novelty phone, gilded seafood cover, mirror selfie trend, iphone 16 pro max, galaxy s25 tough, magsafe phone case, statement phone case, regal aesthetic tech</t>
         </is>
       </c>
     </row>
@@ -7546,15 +7546,15 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #48, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>The Vintage Winding Key Scrollback Sardine Tin Case, Industrial Metal Opener Strip Cover iPhone 16 Pro Max Samsung S25</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>nordic sardine phone case, scandinavian fish tin case, copenhagen aesthetic phone, smoked sprat case, minimalist fish case, danish smorrebrod phone case, baltic herring phone cover, clean scandi phone case, iphone 16 case, samsung s24 case, modern minimalist phone case, architectural graphic case, aesthetic gift</t>
+          <t>winding key tin case, sardine key opener, metal scrollback art, vintage mechanics, retro tin opener, industrial packaging, steampunk food case, novelty tech gift, iphone 16 pro max, samsung s25 ultra, magsafe tough case, tactile metal look, unique phone case</t>
         </is>
       </c>
     </row>
@@ -7564,15 +7564,15 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #49, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Crushed Pop-Art Halftone Dented Sardine Can Case, Retro Streetwear Comic Metal Cover iPhone 16 Pro Max Galaxy S25</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>yacht club phone case, vintage nautical tin case, saint tropez seafood case, riviera sailing phone case, maritime provisions case, monaco grand prix phone, sailing flag phone case, boat lover phone cover, iphone 16 pro max case, samsung s25 tough case, preppy nautical gift, coastal aesthetic phone, magsafe cover</t>
+          <t>crushed tin can case, pop art sardine, halftone comic fish, dented can aesthetic, streetwear phone case, retro grunge metal, andy warhol food art, bold graphic phone, iphone 16 pro max, galaxy s25 tough, magsafe phone cover, indie artist gift, edgy novelty cover</t>
         </is>
       </c>
     </row>
@@ -7582,15 +7582,15 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Funny Cat in Sardine Tin Phone Case #50, Quirky Orange Tabby Seafood Can Bed Cover iPhone 16 15 Pro Max Galaxy S25 Tough Case</t>
+          <t>Transparent Floating Olive Oil &amp; Sardines Phone Case, Clear Back Floating Herb Can iPhone 16 Pro Max Samsung Galaxy S25</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3d sardine tin phone case, peel back tin phone case, metal sardine can case, realistic sardine can case, illusion food case, open tin can phone cover, funny food phone case, realistic 3d food case, iphone 16 pro max case, samsung s25 ultra cover, novelty phone case, viral tiktok phone case, conversation starter</t>
+          <t>clear sardine case, floating olive oil, transparent fish tin, floating rosemary art, clear back cover, minimalist liquid art, viral aesthetic phone, cute foodie accessory, iphone 16 pro max, samsung s25 tough, magsafe phone case, clean phone cover, summer phone trend</t>
         </is>
       </c>
     </row>

</xml_diff>